<commit_message>
fixed data undefined problem
</commit_message>
<xml_diff>
--- a/Week 1/Playwright/data/credit_data.xlsx
+++ b/Week 1/Playwright/data/credit_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\308345\Documents\Testing\Week 1\Playwright\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EF806823-58B9-4C32-BA9E-2028E2B8FAEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BB5818A-9C09-471E-A41F-FB10F816FB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9030BD1D-A4E2-4469-B3D4-144378E2A888}"/>
   </bookViews>
@@ -38,18 +38,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
-    <t>Pan</t>
-  </si>
-  <si>
-    <t>Gender</t>
-  </si>
-  <si>
-    <t>Nationality</t>
-  </si>
-  <si>
-    <t>Mothers Name</t>
-  </si>
-  <si>
     <t>email</t>
   </si>
   <si>
@@ -75,6 +63,18 @@
   </si>
   <si>
     <t>Step 2 of 4</t>
+  </si>
+  <si>
+    <t>pan</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>nationality</t>
+  </si>
+  <si>
+    <t>mother_name</t>
   </si>
 </sst>
 </file>
@@ -483,48 +483,48 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>11</v>
       </c>
       <c r="F2" s="1">
         <v>685552</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H2" s="1"/>
     </row>

</xml_diff>

<commit_message>
added Data Driven Testing
</commit_message>
<xml_diff>
--- a/Week 1/Playwright/data/credit_data.xlsx
+++ b/Week 1/Playwright/data/credit_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\308345\Documents\Testing\Week 1\Playwright\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BB5818A-9C09-471E-A41F-FB10F816FB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BF155E1-9A7B-48B9-A518-DEDF3463C0C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9030BD1D-A4E2-4469-B3D4-144378E2A888}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="22">
   <si>
     <t>email</t>
   </si>
@@ -75,6 +75,33 @@
   </si>
   <si>
     <t>mother_name</t>
+  </si>
+  <si>
+    <t>scenario</t>
+  </si>
+  <si>
+    <t>valid</t>
+  </si>
+  <si>
+    <t>NOPANFORYO</t>
+  </si>
+  <si>
+    <t>invalid</t>
+  </si>
+  <si>
+    <t>PAN not valid, please enter a valid PAN</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>Please enter a valid email ID</t>
+  </si>
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>Please enter a valid mother's name (minimum 3 characters)</t>
   </si>
 </sst>
 </file>
@@ -125,7 +152,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -135,6 +162,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -471,14 +504,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{664EE447-84A1-4799-88F8-D22BAD4843D7}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
     <col min="5" max="5" width="20.6640625" customWidth="1"/>
-    <col min="7" max="7" width="13.5546875" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" customWidth="1"/>
+    <col min="8" max="8" width="13.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -503,6 +537,9 @@
       <c r="G1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -526,11 +563,119 @@
       <c r="G2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="1"/>
+      <c r="H2" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="4">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="4">
+        <v>685552</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="4">
+        <v>685552</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>12</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" xr:uid="{4CF8CC51-1AFB-45BD-8D04-56A15BE91E01}"/>
+    <hyperlink ref="E5" r:id="rId2" xr:uid="{A4E8A26E-748D-4404-AD55-02B2531E371D}"/>
+    <hyperlink ref="E6" r:id="rId3" xr:uid="{0BB17AA0-84B4-465F-B78E-D7BBF397B887}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>